<commit_message>
Additional progress in logging spike-ins.
</commit_message>
<xml_diff>
--- a/analysis/resources/PLATES_v2.0.0/AB[BATCH_ID].3SARS.xlsx
+++ b/analysis/resources/PLATES_v2.0.0/AB[BATCH_ID].3SARS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/analysis/resources/PLATES_v2.0.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45233C66-F0AC-CA43-A429-861D104F22AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3576DF-193E-6148-B803-95BA44026EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,9 +18,8 @@
     <sheet name="Extraction IDs" sheetId="9" r:id="rId3"/>
     <sheet name="Comments" sheetId="4" r:id="rId4"/>
     <sheet name="Volume Overrides" sheetId="8" r:id="rId5"/>
-    <sheet name="Spikes" sheetId="10" r:id="rId6"/>
-    <sheet name="Run Setup" sheetId="2" r:id="rId7"/>
-    <sheet name="Lists" sheetId="5" r:id="rId8"/>
+    <sheet name="Run Setup" sheetId="2" r:id="rId6"/>
+    <sheet name="Lists" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="203">
   <si>
     <t>Assay</t>
   </si>
@@ -491,36 +490,6 @@
     <t>NEP/NS1</t>
   </si>
   <si>
-    <t>Spike-In</t>
-  </si>
-  <si>
-    <t>(Same as target itself)</t>
-  </si>
-  <si>
-    <t>Record for each spiked well on the "Spikes" sheet, as copies/µL reaction of the spike.</t>
-  </si>
-  <si>
-    <t>Spikes</t>
-  </si>
-  <si>
-    <t>Pre-concentration, Biological</t>
-  </si>
-  <si>
-    <t>Pre-concentration, Nucleic Acid</t>
-  </si>
-  <si>
-    <t>Post-concentration, Biological</t>
-  </si>
-  <si>
-    <t>Post-concentration, Nucleic Acid</t>
-  </si>
-  <si>
-    <t>Pre-concentration, Other</t>
-  </si>
-  <si>
-    <t>Post-concentration, Other</t>
-  </si>
-  <si>
     <t>Enterovirus</t>
   </si>
   <si>
@@ -576,12 +545,6 @@
   </si>
   <si>
     <t>C3b</t>
-  </si>
-  <si>
-    <t>Post-extraction, Nucleic Acid</t>
-  </si>
-  <si>
-    <t>Post-extraction, Other</t>
   </si>
   <si>
     <t>SARS-CoV-2 (N1, N2), Human (RNAse P) Triplex (dEXD28563542)</t>
@@ -1213,7 +1176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1419,26 +1382,10 @@
     <xf numFmtId="0" fontId="16" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2118,7 +2065,7 @@
         <v>115</v>
       </c>
       <c r="B14" s="42" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="C14" s="49"/>
       <c r="D14" s="42"/>
@@ -2216,7 +2163,7 @@
       <c r="B17" s="68" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="75"/>
+      <c r="C17"/>
       <c r="E17" s="42"/>
       <c r="F17" s="42"/>
       <c r="G17" s="42"/>
@@ -2247,7 +2194,7 @@
       <c r="B18" s="52" t="s">
         <v>71</v>
       </c>
-      <c r="C18" s="82"/>
+      <c r="C18"/>
       <c r="D18" s="42"/>
       <c r="E18" s="42"/>
       <c r="F18" s="42"/>
@@ -2274,14 +2221,12 @@
     </row>
     <row r="19" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="52" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="B19" s="52" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
-      <c r="C19" s="74" t="s">
-        <v>149</v>
-      </c>
+      <c r="C19"/>
       <c r="D19" s="42"/>
       <c r="E19" s="42"/>
       <c r="F19" s="42"/>
@@ -2311,11 +2256,9 @@
         <v>118</v>
       </c>
       <c r="B20" s="54" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
-      <c r="C20" s="76" t="s">
-        <v>150</v>
-      </c>
+      <c r="C20"/>
     </row>
     <row r="21" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="52" t="s">
@@ -2324,7 +2267,7 @@
       <c r="B21" s="52" t="s">
         <v>98</v>
       </c>
-      <c r="C21" s="73"/>
+      <c r="C21"/>
       <c r="D21" s="42"/>
       <c r="E21" s="42"/>
       <c r="F21" s="42"/>
@@ -2356,7 +2299,7 @@
       <c r="B22" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="73"/>
+      <c r="C22"/>
       <c r="D22" s="42"/>
       <c r="E22" s="42"/>
       <c r="F22" s="42"/>
@@ -2388,9 +2331,7 @@
       <c r="B23" s="52">
         <v>0</v>
       </c>
-      <c r="C23" s="77" t="s">
-        <v>151</v>
-      </c>
+      <c r="C23"/>
       <c r="D23" s="42"/>
       <c r="E23" s="42"/>
       <c r="F23" s="42"/>
@@ -2693,7 +2634,7 @@
       <c r="B34" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="75"/>
+      <c r="C34"/>
       <c r="D34" s="42"/>
       <c r="E34" s="42"/>
       <c r="F34" s="42"/>
@@ -2725,7 +2666,7 @@
       <c r="B35" s="52" t="s">
         <v>71</v>
       </c>
-      <c r="C35" s="74"/>
+      <c r="C35"/>
       <c r="D35" s="42"/>
       <c r="E35" s="42"/>
       <c r="F35" s="42"/>
@@ -2752,14 +2693,12 @@
     </row>
     <row r="36" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="52" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="B36" s="52" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
-      <c r="C36" s="74" t="s">
-        <v>149</v>
-      </c>
+      <c r="C36"/>
       <c r="D36" s="42"/>
       <c r="E36" s="42"/>
       <c r="F36" s="42"/>
@@ -2789,11 +2728,9 @@
         <v>118</v>
       </c>
       <c r="B37" s="54" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
-      <c r="C37" s="76" t="s">
-        <v>150</v>
-      </c>
+      <c r="C37"/>
       <c r="D37" s="42"/>
       <c r="E37" s="42"/>
       <c r="F37" s="42"/>
@@ -2825,7 +2762,7 @@
       <c r="B38" s="52" t="s">
         <v>98</v>
       </c>
-      <c r="C38" s="73"/>
+      <c r="C38"/>
       <c r="D38" s="42"/>
       <c r="E38" s="42"/>
       <c r="F38" s="42"/>
@@ -2857,7 +2794,7 @@
       <c r="B39" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="C39" s="73"/>
+      <c r="C39"/>
       <c r="D39" s="42"/>
       <c r="E39" s="42"/>
       <c r="F39" s="42"/>
@@ -2889,9 +2826,7 @@
       <c r="B40" s="52">
         <v>0</v>
       </c>
-      <c r="C40" s="77" t="s">
-        <v>151</v>
-      </c>
+      <c r="C40"/>
       <c r="D40" s="42"/>
       <c r="E40" s="42"/>
       <c r="F40" s="42"/>
@@ -3239,7 +3174,7 @@
       <c r="B51" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="C51" s="75"/>
+      <c r="C51"/>
       <c r="D51" s="42"/>
       <c r="E51" s="42"/>
       <c r="F51" s="42"/>
@@ -3269,9 +3204,9 @@
         <v>104</v>
       </c>
       <c r="B52" s="52" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
-      <c r="C52" s="74"/>
+      <c r="C52"/>
       <c r="D52" s="42"/>
       <c r="E52" s="42"/>
       <c r="F52" s="42"/>
@@ -3298,14 +3233,12 @@
     </row>
     <row r="53" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="52" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="B53" s="52" t="s">
         <v>140</v>
       </c>
-      <c r="C53" s="74" t="s">
-        <v>149</v>
-      </c>
+      <c r="C53"/>
       <c r="D53" s="42"/>
       <c r="E53" s="42"/>
       <c r="F53" s="42"/>
@@ -3337,9 +3270,7 @@
       <c r="B54" s="54" t="s">
         <v>113</v>
       </c>
-      <c r="C54" s="76" t="s">
-        <v>150</v>
-      </c>
+      <c r="C54"/>
       <c r="D54" s="42"/>
       <c r="E54" s="42"/>
       <c r="F54" s="42"/>
@@ -3371,7 +3302,7 @@
       <c r="B55" s="52" t="s">
         <v>99</v>
       </c>
-      <c r="C55" s="73"/>
+      <c r="C55"/>
       <c r="D55" s="42"/>
       <c r="E55" s="42"/>
       <c r="F55" s="42"/>
@@ -3403,7 +3334,7 @@
       <c r="B56" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="C56" s="73"/>
+      <c r="C56"/>
       <c r="D56" s="42"/>
       <c r="E56" s="42"/>
       <c r="F56" s="42"/>
@@ -3435,9 +3366,7 @@
       <c r="B57" s="52">
         <v>0</v>
       </c>
-      <c r="C57" s="77" t="s">
-        <v>151</v>
-      </c>
+      <c r="C57"/>
       <c r="D57" s="42"/>
       <c r="E57" s="42"/>
       <c r="F57" s="42"/>
@@ -27747,7 +27676,7 @@
   <pageSetup orientation="landscape"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="22">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="21">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9269EC84-DF31-1A4B-A990-FD99E0DF6A37}">
           <x14:formula1>
             <xm:f>Lists!$F$2:$F$10</xm:f>
@@ -27788,7 +27717,7 @@
           <x14:formula1>
             <xm:f>Lists!$E$2:$E$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B26 B31 B43 B48 B39:C39 B60 B65 B56:C56 B22:C22</xm:sqref>
+          <xm:sqref>B26 B31 B43 B48 B22 B60 B65 B39 B56</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{8B68413C-BA2E-3E4F-BCCD-63E54D16131E}">
           <x14:formula1>
@@ -27820,12 +27749,6 @@
           </x14:formula1>
           <xm:sqref>B34 B17 B51</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EE6A7E99-E8C2-2C46-99ED-4766928B6A0B}">
-          <x14:formula1>
-            <xm:f>Lists!$N$3:$N$10</xm:f>
-          </x14:formula1>
-          <xm:sqref>C21 C55 C38</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{209ABDC6-7A4F-1043-BD31-F5067EDD9592}">
           <x14:formula1>
             <xm:f>Lists!$D$2:$D$27</xm:f>
@@ -27840,15 +27763,15 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{458F1957-7F4C-3843-8AFA-688CEDE96E83}">
           <x14:formula1>
-            <xm:f>Lists!$O$2:$O$7</xm:f>
+            <xm:f>Lists!$N$2:$N$7</xm:f>
           </x14:formula1>
-          <xm:sqref>B19 B36 B53</xm:sqref>
+          <xm:sqref>B19 B53 B36</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B241593E-F5D9-0643-9841-833D07C14BE8}">
           <x14:formula1>
-            <xm:f>Lists!$O$2:$O$7</xm:f>
+            <xm:f>Lists!$N$2:$N$7</xm:f>
           </x14:formula1>
-          <xm:sqref>B19 B36 B53</xm:sqref>
+          <xm:sqref>B19 B53 B36</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{970994F8-0C5A-954C-8A5B-082DB9E55E96}">
           <x14:formula1>
@@ -40601,3183 +40524,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEC9D1D4-5508-E34C-A1ED-A24B8133857F}">
-  <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="13" width="20.5703125" customWidth="1"/>
-    <col min="14" max="26" width="11.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:26" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="35"/>
-      <c r="B1" s="35">
-        <v>1</v>
-      </c>
-      <c r="C1" s="35">
-        <v>2</v>
-      </c>
-      <c r="D1" s="35">
-        <v>3</v>
-      </c>
-      <c r="E1" s="35">
-        <v>4</v>
-      </c>
-      <c r="F1" s="35">
-        <v>5</v>
-      </c>
-      <c r="G1" s="35">
-        <v>6</v>
-      </c>
-      <c r="H1" s="35">
-        <v>7</v>
-      </c>
-      <c r="I1" s="35">
-        <v>8</v>
-      </c>
-      <c r="J1" s="35">
-        <v>9</v>
-      </c>
-      <c r="K1" s="35">
-        <v>10</v>
-      </c>
-      <c r="L1" s="35">
-        <v>11</v>
-      </c>
-      <c r="M1" s="35">
-        <v>12</v>
-      </c>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="35"/>
-      <c r="Y1" s="35"/>
-      <c r="Z1" s="35"/>
-    </row>
-    <row r="2" spans="1:26" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="35" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="37"/>
-    </row>
-    <row r="3" spans="1:26" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="35" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="37"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="37"/>
-      <c r="M3" s="36"/>
-    </row>
-    <row r="4" spans="1:26" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="37"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="37"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="37"/>
-    </row>
-    <row r="5" spans="1:26" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="37"/>
-      <c r="M5" s="36"/>
-    </row>
-    <row r="6" spans="1:26" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="35" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="36"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="37"/>
-      <c r="L6" s="36"/>
-      <c r="M6" s="37"/>
-    </row>
-    <row r="7" spans="1:26" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="35" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
-      <c r="K7" s="36"/>
-      <c r="L7" s="37"/>
-      <c r="M7" s="36"/>
-    </row>
-    <row r="8" spans="1:26" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37"/>
-      <c r="J8" s="36"/>
-      <c r="K8" s="37"/>
-      <c r="L8" s="36"/>
-      <c r="M8" s="37"/>
-    </row>
-    <row r="9" spans="1:26" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
-      <c r="K9" s="36"/>
-      <c r="L9" s="37"/>
-      <c r="M9" s="36"/>
-    </row>
-    <row r="10" spans="1:26" ht="31" x14ac:dyDescent="0.2">
-      <c r="A10" s="35"/>
-    </row>
-    <row r="11" spans="1:26" ht="31" x14ac:dyDescent="0.2">
-      <c r="A11" s="35"/>
-    </row>
-    <row r="12" spans="1:26" ht="31" x14ac:dyDescent="0.2">
-      <c r="A12" s="35"/>
-    </row>
-    <row r="13" spans="1:26" ht="31" x14ac:dyDescent="0.2">
-      <c r="A13" s="35"/>
-    </row>
-    <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="35"/>
-    </row>
-    <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="35"/>
-    </row>
-    <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="35"/>
-    </row>
-    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="35"/>
-    </row>
-    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="35"/>
-    </row>
-    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="35"/>
-    </row>
-    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="35"/>
-    </row>
-    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="35"/>
-    </row>
-    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="35"/>
-    </row>
-    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="35"/>
-    </row>
-    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="35"/>
-    </row>
-    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="35"/>
-    </row>
-    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="35"/>
-    </row>
-    <row r="27" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="35"/>
-    </row>
-    <row r="28" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="35"/>
-    </row>
-    <row r="29" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="35"/>
-    </row>
-    <row r="30" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="35"/>
-    </row>
-    <row r="31" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="35"/>
-    </row>
-    <row r="32" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="35"/>
-    </row>
-    <row r="33" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="35"/>
-    </row>
-    <row r="34" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="35"/>
-    </row>
-    <row r="35" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="35"/>
-    </row>
-    <row r="36" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="35"/>
-    </row>
-    <row r="37" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="35"/>
-    </row>
-    <row r="38" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="35"/>
-    </row>
-    <row r="39" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="35"/>
-    </row>
-    <row r="40" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="35"/>
-    </row>
-    <row r="41" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="35"/>
-    </row>
-    <row r="42" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="35"/>
-    </row>
-    <row r="43" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="35"/>
-    </row>
-    <row r="44" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="35"/>
-    </row>
-    <row r="45" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="35"/>
-    </row>
-    <row r="46" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="35"/>
-    </row>
-    <row r="47" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="35"/>
-    </row>
-    <row r="48" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="35"/>
-    </row>
-    <row r="49" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="35"/>
-    </row>
-    <row r="50" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="35"/>
-    </row>
-    <row r="51" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="35"/>
-    </row>
-    <row r="52" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="35"/>
-    </row>
-    <row r="53" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="35"/>
-    </row>
-    <row r="54" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="35"/>
-    </row>
-    <row r="55" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="35"/>
-    </row>
-    <row r="56" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="35"/>
-    </row>
-    <row r="57" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="35"/>
-    </row>
-    <row r="58" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="35"/>
-    </row>
-    <row r="59" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="35"/>
-    </row>
-    <row r="60" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="35"/>
-    </row>
-    <row r="61" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="35"/>
-    </row>
-    <row r="62" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="35"/>
-    </row>
-    <row r="63" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="35"/>
-    </row>
-    <row r="64" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="35"/>
-    </row>
-    <row r="65" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="35"/>
-    </row>
-    <row r="66" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="35"/>
-    </row>
-    <row r="67" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="35"/>
-    </row>
-    <row r="68" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="35"/>
-    </row>
-    <row r="69" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="35"/>
-    </row>
-    <row r="70" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="35"/>
-    </row>
-    <row r="71" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="35"/>
-    </row>
-    <row r="72" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="35"/>
-    </row>
-    <row r="73" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="35"/>
-    </row>
-    <row r="74" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="35"/>
-    </row>
-    <row r="75" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="35"/>
-    </row>
-    <row r="76" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="35"/>
-    </row>
-    <row r="77" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="35"/>
-    </row>
-    <row r="78" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="35"/>
-    </row>
-    <row r="79" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="35"/>
-    </row>
-    <row r="80" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="35"/>
-    </row>
-    <row r="81" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="35"/>
-    </row>
-    <row r="82" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="35"/>
-    </row>
-    <row r="83" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="35"/>
-    </row>
-    <row r="84" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="35"/>
-    </row>
-    <row r="85" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="35"/>
-    </row>
-    <row r="86" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="35"/>
-    </row>
-    <row r="87" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="35"/>
-    </row>
-    <row r="88" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="35"/>
-    </row>
-    <row r="89" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="35"/>
-    </row>
-    <row r="90" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="35"/>
-    </row>
-    <row r="91" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="35"/>
-    </row>
-    <row r="92" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="35"/>
-    </row>
-    <row r="93" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="35"/>
-    </row>
-    <row r="94" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="35"/>
-    </row>
-    <row r="95" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="35"/>
-    </row>
-    <row r="96" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="35"/>
-    </row>
-    <row r="97" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="35"/>
-    </row>
-    <row r="98" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="35"/>
-    </row>
-    <row r="99" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="35"/>
-    </row>
-    <row r="100" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="35"/>
-    </row>
-    <row r="101" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="35"/>
-    </row>
-    <row r="102" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="35"/>
-    </row>
-    <row r="103" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A103" s="35"/>
-    </row>
-    <row r="104" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A104" s="35"/>
-    </row>
-    <row r="105" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A105" s="35"/>
-    </row>
-    <row r="106" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A106" s="35"/>
-    </row>
-    <row r="107" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="35"/>
-    </row>
-    <row r="108" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A108" s="35"/>
-    </row>
-    <row r="109" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="35"/>
-    </row>
-    <row r="110" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="35"/>
-    </row>
-    <row r="111" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A111" s="35"/>
-    </row>
-    <row r="112" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="35"/>
-    </row>
-    <row r="113" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A113" s="35"/>
-    </row>
-    <row r="114" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A114" s="35"/>
-    </row>
-    <row r="115" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A115" s="35"/>
-    </row>
-    <row r="116" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="35"/>
-    </row>
-    <row r="117" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A117" s="35"/>
-    </row>
-    <row r="118" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A118" s="35"/>
-    </row>
-    <row r="119" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="35"/>
-    </row>
-    <row r="120" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A120" s="35"/>
-    </row>
-    <row r="121" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A121" s="35"/>
-    </row>
-    <row r="122" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A122" s="35"/>
-    </row>
-    <row r="123" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="35"/>
-    </row>
-    <row r="124" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="35"/>
-    </row>
-    <row r="125" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="35"/>
-    </row>
-    <row r="126" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="35"/>
-    </row>
-    <row r="127" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="35"/>
-    </row>
-    <row r="128" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="35"/>
-    </row>
-    <row r="129" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="35"/>
-    </row>
-    <row r="130" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" s="35"/>
-    </row>
-    <row r="131" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" s="35"/>
-    </row>
-    <row r="132" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="35"/>
-    </row>
-    <row r="133" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="35"/>
-    </row>
-    <row r="134" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="35"/>
-    </row>
-    <row r="135" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" s="35"/>
-    </row>
-    <row r="136" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A136" s="35"/>
-    </row>
-    <row r="137" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" s="35"/>
-    </row>
-    <row r="138" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="35"/>
-    </row>
-    <row r="139" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" s="35"/>
-    </row>
-    <row r="140" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="35"/>
-    </row>
-    <row r="141" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="35"/>
-    </row>
-    <row r="142" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A142" s="35"/>
-    </row>
-    <row r="143" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="35"/>
-    </row>
-    <row r="144" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="35"/>
-    </row>
-    <row r="145" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="35"/>
-    </row>
-    <row r="146" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="35"/>
-    </row>
-    <row r="147" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="35"/>
-    </row>
-    <row r="148" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="35"/>
-    </row>
-    <row r="149" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="35"/>
-    </row>
-    <row r="150" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="35"/>
-    </row>
-    <row r="151" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="35"/>
-    </row>
-    <row r="152" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="35"/>
-    </row>
-    <row r="153" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="35"/>
-    </row>
-    <row r="154" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="35"/>
-    </row>
-    <row r="155" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="35"/>
-    </row>
-    <row r="156" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="35"/>
-    </row>
-    <row r="157" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="35"/>
-    </row>
-    <row r="158" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="35"/>
-    </row>
-    <row r="159" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="35"/>
-    </row>
-    <row r="160" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="35"/>
-    </row>
-    <row r="161" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="35"/>
-    </row>
-    <row r="162" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="35"/>
-    </row>
-    <row r="163" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="35"/>
-    </row>
-    <row r="164" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="35"/>
-    </row>
-    <row r="165" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="35"/>
-    </row>
-    <row r="166" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="35"/>
-    </row>
-    <row r="167" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A167" s="35"/>
-    </row>
-    <row r="168" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="35"/>
-    </row>
-    <row r="169" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A169" s="35"/>
-    </row>
-    <row r="170" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A170" s="35"/>
-    </row>
-    <row r="171" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A171" s="35"/>
-    </row>
-    <row r="172" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A172" s="35"/>
-    </row>
-    <row r="173" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A173" s="35"/>
-    </row>
-    <row r="174" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A174" s="35"/>
-    </row>
-    <row r="175" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A175" s="35"/>
-    </row>
-    <row r="176" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A176" s="35"/>
-    </row>
-    <row r="177" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A177" s="35"/>
-    </row>
-    <row r="178" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A178" s="35"/>
-    </row>
-    <row r="179" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A179" s="35"/>
-    </row>
-    <row r="180" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A180" s="35"/>
-    </row>
-    <row r="181" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A181" s="35"/>
-    </row>
-    <row r="182" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A182" s="35"/>
-    </row>
-    <row r="183" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A183" s="35"/>
-    </row>
-    <row r="184" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A184" s="35"/>
-    </row>
-    <row r="185" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A185" s="35"/>
-    </row>
-    <row r="186" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A186" s="35"/>
-    </row>
-    <row r="187" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A187" s="35"/>
-    </row>
-    <row r="188" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A188" s="35"/>
-    </row>
-    <row r="189" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A189" s="35"/>
-    </row>
-    <row r="190" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A190" s="35"/>
-    </row>
-    <row r="191" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A191" s="35"/>
-    </row>
-    <row r="192" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A192" s="35"/>
-    </row>
-    <row r="193" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A193" s="35"/>
-    </row>
-    <row r="194" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A194" s="35"/>
-    </row>
-    <row r="195" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A195" s="35"/>
-    </row>
-    <row r="196" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A196" s="35"/>
-    </row>
-    <row r="197" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A197" s="35"/>
-    </row>
-    <row r="198" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A198" s="35"/>
-    </row>
-    <row r="199" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A199" s="35"/>
-    </row>
-    <row r="200" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A200" s="35"/>
-    </row>
-    <row r="201" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A201" s="35"/>
-    </row>
-    <row r="202" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A202" s="35"/>
-    </row>
-    <row r="203" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A203" s="35"/>
-    </row>
-    <row r="204" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A204" s="35"/>
-    </row>
-    <row r="205" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A205" s="35"/>
-    </row>
-    <row r="206" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A206" s="35"/>
-    </row>
-    <row r="207" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A207" s="35"/>
-    </row>
-    <row r="208" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A208" s="35"/>
-    </row>
-    <row r="209" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A209" s="35"/>
-    </row>
-    <row r="210" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A210" s="35"/>
-    </row>
-    <row r="211" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A211" s="35"/>
-    </row>
-    <row r="212" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A212" s="35"/>
-    </row>
-    <row r="213" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A213" s="35"/>
-    </row>
-    <row r="214" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A214" s="35"/>
-    </row>
-    <row r="215" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A215" s="35"/>
-    </row>
-    <row r="216" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A216" s="35"/>
-    </row>
-    <row r="217" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A217" s="35"/>
-    </row>
-    <row r="218" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A218" s="35"/>
-    </row>
-    <row r="219" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A219" s="35"/>
-    </row>
-    <row r="220" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A220" s="35"/>
-    </row>
-    <row r="221" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A221" s="35"/>
-    </row>
-    <row r="222" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A222" s="35"/>
-    </row>
-    <row r="223" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A223" s="35"/>
-    </row>
-    <row r="224" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A224" s="35"/>
-    </row>
-    <row r="225" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A225" s="35"/>
-    </row>
-    <row r="226" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A226" s="35"/>
-    </row>
-    <row r="227" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A227" s="35"/>
-    </row>
-    <row r="228" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A228" s="35"/>
-    </row>
-    <row r="229" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A229" s="35"/>
-    </row>
-    <row r="230" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A230" s="35"/>
-    </row>
-    <row r="231" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A231" s="35"/>
-    </row>
-    <row r="232" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A232" s="35"/>
-    </row>
-    <row r="233" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A233" s="35"/>
-    </row>
-    <row r="234" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A234" s="35"/>
-    </row>
-    <row r="235" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A235" s="35"/>
-    </row>
-    <row r="236" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A236" s="35"/>
-    </row>
-    <row r="237" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A237" s="35"/>
-    </row>
-    <row r="238" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A238" s="35"/>
-    </row>
-    <row r="239" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A239" s="35"/>
-    </row>
-    <row r="240" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A240" s="35"/>
-    </row>
-    <row r="241" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A241" s="35"/>
-    </row>
-    <row r="242" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A242" s="35"/>
-    </row>
-    <row r="243" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A243" s="35"/>
-    </row>
-    <row r="244" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A244" s="35"/>
-    </row>
-    <row r="245" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A245" s="35"/>
-    </row>
-    <row r="246" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A246" s="35"/>
-    </row>
-    <row r="247" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A247" s="35"/>
-    </row>
-    <row r="248" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A248" s="35"/>
-    </row>
-    <row r="249" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A249" s="35"/>
-    </row>
-    <row r="250" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A250" s="35"/>
-    </row>
-    <row r="251" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A251" s="35"/>
-    </row>
-    <row r="252" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A252" s="35"/>
-    </row>
-    <row r="253" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A253" s="35"/>
-    </row>
-    <row r="254" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A254" s="35"/>
-    </row>
-    <row r="255" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A255" s="35"/>
-    </row>
-    <row r="256" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A256" s="35"/>
-    </row>
-    <row r="257" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A257" s="35"/>
-    </row>
-    <row r="258" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A258" s="35"/>
-    </row>
-    <row r="259" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A259" s="35"/>
-    </row>
-    <row r="260" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A260" s="35"/>
-    </row>
-    <row r="261" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A261" s="35"/>
-    </row>
-    <row r="262" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A262" s="35"/>
-    </row>
-    <row r="263" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A263" s="35"/>
-    </row>
-    <row r="264" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A264" s="35"/>
-    </row>
-    <row r="265" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A265" s="35"/>
-    </row>
-    <row r="266" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A266" s="35"/>
-    </row>
-    <row r="267" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A267" s="35"/>
-    </row>
-    <row r="268" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A268" s="35"/>
-    </row>
-    <row r="269" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A269" s="35"/>
-    </row>
-    <row r="270" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A270" s="35"/>
-    </row>
-    <row r="271" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A271" s="35"/>
-    </row>
-    <row r="272" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A272" s="35"/>
-    </row>
-    <row r="273" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A273" s="35"/>
-    </row>
-    <row r="274" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A274" s="35"/>
-    </row>
-    <row r="275" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A275" s="35"/>
-    </row>
-    <row r="276" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A276" s="35"/>
-    </row>
-    <row r="277" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A277" s="35"/>
-    </row>
-    <row r="278" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A278" s="35"/>
-    </row>
-    <row r="279" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A279" s="35"/>
-    </row>
-    <row r="280" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A280" s="35"/>
-    </row>
-    <row r="281" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A281" s="35"/>
-    </row>
-    <row r="282" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A282" s="35"/>
-    </row>
-    <row r="283" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A283" s="35"/>
-    </row>
-    <row r="284" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A284" s="35"/>
-    </row>
-    <row r="285" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A285" s="35"/>
-    </row>
-    <row r="286" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A286" s="35"/>
-    </row>
-    <row r="287" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A287" s="35"/>
-    </row>
-    <row r="288" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A288" s="35"/>
-    </row>
-    <row r="289" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A289" s="35"/>
-    </row>
-    <row r="290" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A290" s="35"/>
-    </row>
-    <row r="291" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A291" s="35"/>
-    </row>
-    <row r="292" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A292" s="35"/>
-    </row>
-    <row r="293" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A293" s="35"/>
-    </row>
-    <row r="294" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A294" s="35"/>
-    </row>
-    <row r="295" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A295" s="35"/>
-    </row>
-    <row r="296" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A296" s="35"/>
-    </row>
-    <row r="297" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A297" s="35"/>
-    </row>
-    <row r="298" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A298" s="35"/>
-    </row>
-    <row r="299" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A299" s="35"/>
-    </row>
-    <row r="300" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A300" s="35"/>
-    </row>
-    <row r="301" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A301" s="35"/>
-    </row>
-    <row r="302" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A302" s="35"/>
-    </row>
-    <row r="303" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A303" s="35"/>
-    </row>
-    <row r="304" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A304" s="35"/>
-    </row>
-    <row r="305" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A305" s="35"/>
-    </row>
-    <row r="306" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A306" s="35"/>
-    </row>
-    <row r="307" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A307" s="35"/>
-    </row>
-    <row r="308" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A308" s="35"/>
-    </row>
-    <row r="309" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A309" s="35"/>
-    </row>
-    <row r="310" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A310" s="35"/>
-    </row>
-    <row r="311" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A311" s="35"/>
-    </row>
-    <row r="312" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A312" s="35"/>
-    </row>
-    <row r="313" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A313" s="35"/>
-    </row>
-    <row r="314" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A314" s="35"/>
-    </row>
-    <row r="315" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A315" s="35"/>
-    </row>
-    <row r="316" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A316" s="35"/>
-    </row>
-    <row r="317" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A317" s="35"/>
-    </row>
-    <row r="318" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A318" s="35"/>
-    </row>
-    <row r="319" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A319" s="35"/>
-    </row>
-    <row r="320" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A320" s="35"/>
-    </row>
-    <row r="321" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A321" s="35"/>
-    </row>
-    <row r="322" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A322" s="35"/>
-    </row>
-    <row r="323" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A323" s="35"/>
-    </row>
-    <row r="324" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A324" s="35"/>
-    </row>
-    <row r="325" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A325" s="35"/>
-    </row>
-    <row r="326" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A326" s="35"/>
-    </row>
-    <row r="327" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A327" s="35"/>
-    </row>
-    <row r="328" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A328" s="35"/>
-    </row>
-    <row r="329" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A329" s="35"/>
-    </row>
-    <row r="330" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A330" s="35"/>
-    </row>
-    <row r="331" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A331" s="35"/>
-    </row>
-    <row r="332" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A332" s="35"/>
-    </row>
-    <row r="333" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A333" s="35"/>
-    </row>
-    <row r="334" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A334" s="35"/>
-    </row>
-    <row r="335" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A335" s="35"/>
-    </row>
-    <row r="336" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A336" s="35"/>
-    </row>
-    <row r="337" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A337" s="35"/>
-    </row>
-    <row r="338" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A338" s="35"/>
-    </row>
-    <row r="339" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A339" s="35"/>
-    </row>
-    <row r="340" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A340" s="35"/>
-    </row>
-    <row r="341" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A341" s="35"/>
-    </row>
-    <row r="342" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A342" s="35"/>
-    </row>
-    <row r="343" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A343" s="35"/>
-    </row>
-    <row r="344" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A344" s="35"/>
-    </row>
-    <row r="345" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A345" s="35"/>
-    </row>
-    <row r="346" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A346" s="35"/>
-    </row>
-    <row r="347" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A347" s="35"/>
-    </row>
-    <row r="348" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A348" s="35"/>
-    </row>
-    <row r="349" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A349" s="35"/>
-    </row>
-    <row r="350" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A350" s="35"/>
-    </row>
-    <row r="351" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A351" s="35"/>
-    </row>
-    <row r="352" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A352" s="35"/>
-    </row>
-    <row r="353" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A353" s="35"/>
-    </row>
-    <row r="354" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A354" s="35"/>
-    </row>
-    <row r="355" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A355" s="35"/>
-    </row>
-    <row r="356" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A356" s="35"/>
-    </row>
-    <row r="357" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A357" s="35"/>
-    </row>
-    <row r="358" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A358" s="35"/>
-    </row>
-    <row r="359" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A359" s="35"/>
-    </row>
-    <row r="360" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A360" s="35"/>
-    </row>
-    <row r="361" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A361" s="35"/>
-    </row>
-    <row r="362" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A362" s="35"/>
-    </row>
-    <row r="363" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A363" s="35"/>
-    </row>
-    <row r="364" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A364" s="35"/>
-    </row>
-    <row r="365" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A365" s="35"/>
-    </row>
-    <row r="366" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A366" s="35"/>
-    </row>
-    <row r="367" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A367" s="35"/>
-    </row>
-    <row r="368" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A368" s="35"/>
-    </row>
-    <row r="369" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A369" s="35"/>
-    </row>
-    <row r="370" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A370" s="35"/>
-    </row>
-    <row r="371" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A371" s="35"/>
-    </row>
-    <row r="372" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A372" s="35"/>
-    </row>
-    <row r="373" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A373" s="35"/>
-    </row>
-    <row r="374" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A374" s="35"/>
-    </row>
-    <row r="375" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A375" s="35"/>
-    </row>
-    <row r="376" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A376" s="35"/>
-    </row>
-    <row r="377" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A377" s="35"/>
-    </row>
-    <row r="378" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A378" s="35"/>
-    </row>
-    <row r="379" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A379" s="35"/>
-    </row>
-    <row r="380" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A380" s="35"/>
-    </row>
-    <row r="381" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A381" s="35"/>
-    </row>
-    <row r="382" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A382" s="35"/>
-    </row>
-    <row r="383" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A383" s="35"/>
-    </row>
-    <row r="384" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A384" s="35"/>
-    </row>
-    <row r="385" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A385" s="35"/>
-    </row>
-    <row r="386" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A386" s="35"/>
-    </row>
-    <row r="387" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A387" s="35"/>
-    </row>
-    <row r="388" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A388" s="35"/>
-    </row>
-    <row r="389" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A389" s="35"/>
-    </row>
-    <row r="390" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A390" s="35"/>
-    </row>
-    <row r="391" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A391" s="35"/>
-    </row>
-    <row r="392" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A392" s="35"/>
-    </row>
-    <row r="393" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A393" s="35"/>
-    </row>
-    <row r="394" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A394" s="35"/>
-    </row>
-    <row r="395" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A395" s="35"/>
-    </row>
-    <row r="396" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A396" s="35"/>
-    </row>
-    <row r="397" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A397" s="35"/>
-    </row>
-    <row r="398" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A398" s="35"/>
-    </row>
-    <row r="399" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A399" s="35"/>
-    </row>
-    <row r="400" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A400" s="35"/>
-    </row>
-    <row r="401" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A401" s="35"/>
-    </row>
-    <row r="402" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A402" s="35"/>
-    </row>
-    <row r="403" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A403" s="35"/>
-    </row>
-    <row r="404" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A404" s="35"/>
-    </row>
-    <row r="405" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A405" s="35"/>
-    </row>
-    <row r="406" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A406" s="35"/>
-    </row>
-    <row r="407" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A407" s="35"/>
-    </row>
-    <row r="408" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A408" s="35"/>
-    </row>
-    <row r="409" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A409" s="35"/>
-    </row>
-    <row r="410" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A410" s="35"/>
-    </row>
-    <row r="411" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A411" s="35"/>
-    </row>
-    <row r="412" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A412" s="35"/>
-    </row>
-    <row r="413" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A413" s="35"/>
-    </row>
-    <row r="414" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A414" s="35"/>
-    </row>
-    <row r="415" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A415" s="35"/>
-    </row>
-    <row r="416" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A416" s="35"/>
-    </row>
-    <row r="417" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A417" s="35"/>
-    </row>
-    <row r="418" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A418" s="35"/>
-    </row>
-    <row r="419" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A419" s="35"/>
-    </row>
-    <row r="420" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A420" s="35"/>
-    </row>
-    <row r="421" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A421" s="35"/>
-    </row>
-    <row r="422" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A422" s="35"/>
-    </row>
-    <row r="423" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A423" s="35"/>
-    </row>
-    <row r="424" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A424" s="35"/>
-    </row>
-    <row r="425" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A425" s="35"/>
-    </row>
-    <row r="426" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A426" s="35"/>
-    </row>
-    <row r="427" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A427" s="35"/>
-    </row>
-    <row r="428" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A428" s="35"/>
-    </row>
-    <row r="429" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A429" s="35"/>
-    </row>
-    <row r="430" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A430" s="35"/>
-    </row>
-    <row r="431" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A431" s="35"/>
-    </row>
-    <row r="432" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A432" s="35"/>
-    </row>
-    <row r="433" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A433" s="35"/>
-    </row>
-    <row r="434" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A434" s="35"/>
-    </row>
-    <row r="435" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A435" s="35"/>
-    </row>
-    <row r="436" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A436" s="35"/>
-    </row>
-    <row r="437" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A437" s="35"/>
-    </row>
-    <row r="438" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A438" s="35"/>
-    </row>
-    <row r="439" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A439" s="35"/>
-    </row>
-    <row r="440" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A440" s="35"/>
-    </row>
-    <row r="441" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A441" s="35"/>
-    </row>
-    <row r="442" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A442" s="35"/>
-    </row>
-    <row r="443" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A443" s="35"/>
-    </row>
-    <row r="444" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A444" s="35"/>
-    </row>
-    <row r="445" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A445" s="35"/>
-    </row>
-    <row r="446" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A446" s="35"/>
-    </row>
-    <row r="447" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A447" s="35"/>
-    </row>
-    <row r="448" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A448" s="35"/>
-    </row>
-    <row r="449" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A449" s="35"/>
-    </row>
-    <row r="450" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A450" s="35"/>
-    </row>
-    <row r="451" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A451" s="35"/>
-    </row>
-    <row r="452" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A452" s="35"/>
-    </row>
-    <row r="453" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A453" s="35"/>
-    </row>
-    <row r="454" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A454" s="35"/>
-    </row>
-    <row r="455" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A455" s="35"/>
-    </row>
-    <row r="456" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A456" s="35"/>
-    </row>
-    <row r="457" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A457" s="35"/>
-    </row>
-    <row r="458" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A458" s="35"/>
-    </row>
-    <row r="459" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A459" s="35"/>
-    </row>
-    <row r="460" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A460" s="35"/>
-    </row>
-    <row r="461" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A461" s="35"/>
-    </row>
-    <row r="462" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A462" s="35"/>
-    </row>
-    <row r="463" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A463" s="35"/>
-    </row>
-    <row r="464" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A464" s="35"/>
-    </row>
-    <row r="465" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A465" s="35"/>
-    </row>
-    <row r="466" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A466" s="35"/>
-    </row>
-    <row r="467" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A467" s="35"/>
-    </row>
-    <row r="468" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A468" s="35"/>
-    </row>
-    <row r="469" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A469" s="35"/>
-    </row>
-    <row r="470" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A470" s="35"/>
-    </row>
-    <row r="471" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A471" s="35"/>
-    </row>
-    <row r="472" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A472" s="35"/>
-    </row>
-    <row r="473" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A473" s="35"/>
-    </row>
-    <row r="474" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A474" s="35"/>
-    </row>
-    <row r="475" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A475" s="35"/>
-    </row>
-    <row r="476" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A476" s="35"/>
-    </row>
-    <row r="477" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A477" s="35"/>
-    </row>
-    <row r="478" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A478" s="35"/>
-    </row>
-    <row r="479" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A479" s="35"/>
-    </row>
-    <row r="480" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A480" s="35"/>
-    </row>
-    <row r="481" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A481" s="35"/>
-    </row>
-    <row r="482" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A482" s="35"/>
-    </row>
-    <row r="483" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A483" s="35"/>
-    </row>
-    <row r="484" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A484" s="35"/>
-    </row>
-    <row r="485" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A485" s="35"/>
-    </row>
-    <row r="486" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A486" s="35"/>
-    </row>
-    <row r="487" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A487" s="35"/>
-    </row>
-    <row r="488" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A488" s="35"/>
-    </row>
-    <row r="489" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A489" s="35"/>
-    </row>
-    <row r="490" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A490" s="35"/>
-    </row>
-    <row r="491" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A491" s="35"/>
-    </row>
-    <row r="492" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A492" s="35"/>
-    </row>
-    <row r="493" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A493" s="35"/>
-    </row>
-    <row r="494" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A494" s="35"/>
-    </row>
-    <row r="495" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A495" s="35"/>
-    </row>
-    <row r="496" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A496" s="35"/>
-    </row>
-    <row r="497" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A497" s="35"/>
-    </row>
-    <row r="498" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A498" s="35"/>
-    </row>
-    <row r="499" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A499" s="35"/>
-    </row>
-    <row r="500" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A500" s="35"/>
-    </row>
-    <row r="501" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A501" s="35"/>
-    </row>
-    <row r="502" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A502" s="35"/>
-    </row>
-    <row r="503" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A503" s="35"/>
-    </row>
-    <row r="504" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A504" s="35"/>
-    </row>
-    <row r="505" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A505" s="35"/>
-    </row>
-    <row r="506" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A506" s="35"/>
-    </row>
-    <row r="507" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A507" s="35"/>
-    </row>
-    <row r="508" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A508" s="35"/>
-    </row>
-    <row r="509" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A509" s="35"/>
-    </row>
-    <row r="510" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A510" s="35"/>
-    </row>
-    <row r="511" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A511" s="35"/>
-    </row>
-    <row r="512" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A512" s="35"/>
-    </row>
-    <row r="513" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A513" s="35"/>
-    </row>
-    <row r="514" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A514" s="35"/>
-    </row>
-    <row r="515" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A515" s="35"/>
-    </row>
-    <row r="516" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A516" s="35"/>
-    </row>
-    <row r="517" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A517" s="35"/>
-    </row>
-    <row r="518" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A518" s="35"/>
-    </row>
-    <row r="519" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A519" s="35"/>
-    </row>
-    <row r="520" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A520" s="35"/>
-    </row>
-    <row r="521" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A521" s="35"/>
-    </row>
-    <row r="522" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A522" s="35"/>
-    </row>
-    <row r="523" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A523" s="35"/>
-    </row>
-    <row r="524" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A524" s="35"/>
-    </row>
-    <row r="525" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A525" s="35"/>
-    </row>
-    <row r="526" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A526" s="35"/>
-    </row>
-    <row r="527" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A527" s="35"/>
-    </row>
-    <row r="528" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A528" s="35"/>
-    </row>
-    <row r="529" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A529" s="35"/>
-    </row>
-    <row r="530" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A530" s="35"/>
-    </row>
-    <row r="531" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A531" s="35"/>
-    </row>
-    <row r="532" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A532" s="35"/>
-    </row>
-    <row r="533" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A533" s="35"/>
-    </row>
-    <row r="534" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A534" s="35"/>
-    </row>
-    <row r="535" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A535" s="35"/>
-    </row>
-    <row r="536" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A536" s="35"/>
-    </row>
-    <row r="537" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A537" s="35"/>
-    </row>
-    <row r="538" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A538" s="35"/>
-    </row>
-    <row r="539" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A539" s="35"/>
-    </row>
-    <row r="540" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A540" s="35"/>
-    </row>
-    <row r="541" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A541" s="35"/>
-    </row>
-    <row r="542" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A542" s="35"/>
-    </row>
-    <row r="543" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A543" s="35"/>
-    </row>
-    <row r="544" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A544" s="35"/>
-    </row>
-    <row r="545" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A545" s="35"/>
-    </row>
-    <row r="546" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A546" s="35"/>
-    </row>
-    <row r="547" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A547" s="35"/>
-    </row>
-    <row r="548" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A548" s="35"/>
-    </row>
-    <row r="549" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A549" s="35"/>
-    </row>
-    <row r="550" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A550" s="35"/>
-    </row>
-    <row r="551" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A551" s="35"/>
-    </row>
-    <row r="552" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A552" s="35"/>
-    </row>
-    <row r="553" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A553" s="35"/>
-    </row>
-    <row r="554" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A554" s="35"/>
-    </row>
-    <row r="555" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A555" s="35"/>
-    </row>
-    <row r="556" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A556" s="35"/>
-    </row>
-    <row r="557" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A557" s="35"/>
-    </row>
-    <row r="558" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A558" s="35"/>
-    </row>
-    <row r="559" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A559" s="35"/>
-    </row>
-    <row r="560" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A560" s="35"/>
-    </row>
-    <row r="561" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A561" s="35"/>
-    </row>
-    <row r="562" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A562" s="35"/>
-    </row>
-    <row r="563" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A563" s="35"/>
-    </row>
-    <row r="564" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A564" s="35"/>
-    </row>
-    <row r="565" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A565" s="35"/>
-    </row>
-    <row r="566" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A566" s="35"/>
-    </row>
-    <row r="567" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A567" s="35"/>
-    </row>
-    <row r="568" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A568" s="35"/>
-    </row>
-    <row r="569" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A569" s="35"/>
-    </row>
-    <row r="570" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A570" s="35"/>
-    </row>
-    <row r="571" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A571" s="35"/>
-    </row>
-    <row r="572" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A572" s="35"/>
-    </row>
-    <row r="573" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A573" s="35"/>
-    </row>
-    <row r="574" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A574" s="35"/>
-    </row>
-    <row r="575" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A575" s="35"/>
-    </row>
-    <row r="576" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A576" s="35"/>
-    </row>
-    <row r="577" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A577" s="35"/>
-    </row>
-    <row r="578" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A578" s="35"/>
-    </row>
-    <row r="579" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A579" s="35"/>
-    </row>
-    <row r="580" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A580" s="35"/>
-    </row>
-    <row r="581" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A581" s="35"/>
-    </row>
-    <row r="582" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A582" s="35"/>
-    </row>
-    <row r="583" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A583" s="35"/>
-    </row>
-    <row r="584" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A584" s="35"/>
-    </row>
-    <row r="585" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A585" s="35"/>
-    </row>
-    <row r="586" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A586" s="35"/>
-    </row>
-    <row r="587" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A587" s="35"/>
-    </row>
-    <row r="588" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A588" s="35"/>
-    </row>
-    <row r="589" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A589" s="35"/>
-    </row>
-    <row r="590" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A590" s="35"/>
-    </row>
-    <row r="591" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A591" s="35"/>
-    </row>
-    <row r="592" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A592" s="35"/>
-    </row>
-    <row r="593" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A593" s="35"/>
-    </row>
-    <row r="594" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A594" s="35"/>
-    </row>
-    <row r="595" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A595" s="35"/>
-    </row>
-    <row r="596" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A596" s="35"/>
-    </row>
-    <row r="597" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A597" s="35"/>
-    </row>
-    <row r="598" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A598" s="35"/>
-    </row>
-    <row r="599" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A599" s="35"/>
-    </row>
-    <row r="600" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A600" s="35"/>
-    </row>
-    <row r="601" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A601" s="35"/>
-    </row>
-    <row r="602" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A602" s="35"/>
-    </row>
-    <row r="603" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A603" s="35"/>
-    </row>
-    <row r="604" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A604" s="35"/>
-    </row>
-    <row r="605" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A605" s="35"/>
-    </row>
-    <row r="606" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A606" s="35"/>
-    </row>
-    <row r="607" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A607" s="35"/>
-    </row>
-    <row r="608" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A608" s="35"/>
-    </row>
-    <row r="609" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A609" s="35"/>
-    </row>
-    <row r="610" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A610" s="35"/>
-    </row>
-    <row r="611" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A611" s="35"/>
-    </row>
-    <row r="612" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A612" s="35"/>
-    </row>
-    <row r="613" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A613" s="35"/>
-    </row>
-    <row r="614" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A614" s="35"/>
-    </row>
-    <row r="615" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A615" s="35"/>
-    </row>
-    <row r="616" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A616" s="35"/>
-    </row>
-    <row r="617" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A617" s="35"/>
-    </row>
-    <row r="618" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A618" s="35"/>
-    </row>
-    <row r="619" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A619" s="35"/>
-    </row>
-    <row r="620" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A620" s="35"/>
-    </row>
-    <row r="621" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A621" s="35"/>
-    </row>
-    <row r="622" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A622" s="35"/>
-    </row>
-    <row r="623" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A623" s="35"/>
-    </row>
-    <row r="624" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A624" s="35"/>
-    </row>
-    <row r="625" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A625" s="35"/>
-    </row>
-    <row r="626" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A626" s="35"/>
-    </row>
-    <row r="627" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A627" s="35"/>
-    </row>
-    <row r="628" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A628" s="35"/>
-    </row>
-    <row r="629" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A629" s="35"/>
-    </row>
-    <row r="630" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A630" s="35"/>
-    </row>
-    <row r="631" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A631" s="35"/>
-    </row>
-    <row r="632" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A632" s="35"/>
-    </row>
-    <row r="633" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A633" s="35"/>
-    </row>
-    <row r="634" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A634" s="35"/>
-    </row>
-    <row r="635" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A635" s="35"/>
-    </row>
-    <row r="636" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A636" s="35"/>
-    </row>
-    <row r="637" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A637" s="35"/>
-    </row>
-    <row r="638" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A638" s="35"/>
-    </row>
-    <row r="639" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A639" s="35"/>
-    </row>
-    <row r="640" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A640" s="35"/>
-    </row>
-    <row r="641" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A641" s="35"/>
-    </row>
-    <row r="642" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A642" s="35"/>
-    </row>
-    <row r="643" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A643" s="35"/>
-    </row>
-    <row r="644" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A644" s="35"/>
-    </row>
-    <row r="645" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A645" s="35"/>
-    </row>
-    <row r="646" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A646" s="35"/>
-    </row>
-    <row r="647" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A647" s="35"/>
-    </row>
-    <row r="648" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A648" s="35"/>
-    </row>
-    <row r="649" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A649" s="35"/>
-    </row>
-    <row r="650" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A650" s="35"/>
-    </row>
-    <row r="651" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A651" s="35"/>
-    </row>
-    <row r="652" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A652" s="35"/>
-    </row>
-    <row r="653" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A653" s="35"/>
-    </row>
-    <row r="654" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A654" s="35"/>
-    </row>
-    <row r="655" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A655" s="35"/>
-    </row>
-    <row r="656" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A656" s="35"/>
-    </row>
-    <row r="657" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A657" s="35"/>
-    </row>
-    <row r="658" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A658" s="35"/>
-    </row>
-    <row r="659" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A659" s="35"/>
-    </row>
-    <row r="660" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A660" s="35"/>
-    </row>
-    <row r="661" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A661" s="35"/>
-    </row>
-    <row r="662" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A662" s="35"/>
-    </row>
-    <row r="663" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A663" s="35"/>
-    </row>
-    <row r="664" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A664" s="35"/>
-    </row>
-    <row r="665" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A665" s="35"/>
-    </row>
-    <row r="666" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A666" s="35"/>
-    </row>
-    <row r="667" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A667" s="35"/>
-    </row>
-    <row r="668" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A668" s="35"/>
-    </row>
-    <row r="669" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A669" s="35"/>
-    </row>
-    <row r="670" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A670" s="35"/>
-    </row>
-    <row r="671" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A671" s="35"/>
-    </row>
-    <row r="672" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A672" s="35"/>
-    </row>
-    <row r="673" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A673" s="35"/>
-    </row>
-    <row r="674" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A674" s="35"/>
-    </row>
-    <row r="675" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A675" s="35"/>
-    </row>
-    <row r="676" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A676" s="35"/>
-    </row>
-    <row r="677" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A677" s="35"/>
-    </row>
-    <row r="678" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A678" s="35"/>
-    </row>
-    <row r="679" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A679" s="35"/>
-    </row>
-    <row r="680" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A680" s="35"/>
-    </row>
-    <row r="681" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A681" s="35"/>
-    </row>
-    <row r="682" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A682" s="35"/>
-    </row>
-    <row r="683" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A683" s="35"/>
-    </row>
-    <row r="684" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A684" s="35"/>
-    </row>
-    <row r="685" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A685" s="35"/>
-    </row>
-    <row r="686" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A686" s="35"/>
-    </row>
-    <row r="687" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A687" s="35"/>
-    </row>
-    <row r="688" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A688" s="35"/>
-    </row>
-    <row r="689" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A689" s="35"/>
-    </row>
-    <row r="690" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A690" s="35"/>
-    </row>
-    <row r="691" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A691" s="35"/>
-    </row>
-    <row r="692" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A692" s="35"/>
-    </row>
-    <row r="693" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A693" s="35"/>
-    </row>
-    <row r="694" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A694" s="35"/>
-    </row>
-    <row r="695" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A695" s="35"/>
-    </row>
-    <row r="696" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A696" s="35"/>
-    </row>
-    <row r="697" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A697" s="35"/>
-    </row>
-    <row r="698" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A698" s="35"/>
-    </row>
-    <row r="699" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A699" s="35"/>
-    </row>
-    <row r="700" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A700" s="35"/>
-    </row>
-    <row r="701" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A701" s="35"/>
-    </row>
-    <row r="702" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A702" s="35"/>
-    </row>
-    <row r="703" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A703" s="35"/>
-    </row>
-    <row r="704" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A704" s="35"/>
-    </row>
-    <row r="705" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A705" s="35"/>
-    </row>
-    <row r="706" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A706" s="35"/>
-    </row>
-    <row r="707" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A707" s="35"/>
-    </row>
-    <row r="708" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A708" s="35"/>
-    </row>
-    <row r="709" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A709" s="35"/>
-    </row>
-    <row r="710" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A710" s="35"/>
-    </row>
-    <row r="711" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A711" s="35"/>
-    </row>
-    <row r="712" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A712" s="35"/>
-    </row>
-    <row r="713" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A713" s="35"/>
-    </row>
-    <row r="714" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A714" s="35"/>
-    </row>
-    <row r="715" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A715" s="35"/>
-    </row>
-    <row r="716" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A716" s="35"/>
-    </row>
-    <row r="717" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A717" s="35"/>
-    </row>
-    <row r="718" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A718" s="35"/>
-    </row>
-    <row r="719" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A719" s="35"/>
-    </row>
-    <row r="720" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A720" s="35"/>
-    </row>
-    <row r="721" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A721" s="35"/>
-    </row>
-    <row r="722" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A722" s="35"/>
-    </row>
-    <row r="723" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A723" s="35"/>
-    </row>
-    <row r="724" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A724" s="35"/>
-    </row>
-    <row r="725" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A725" s="35"/>
-    </row>
-    <row r="726" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A726" s="35"/>
-    </row>
-    <row r="727" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A727" s="35"/>
-    </row>
-    <row r="728" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A728" s="35"/>
-    </row>
-    <row r="729" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A729" s="35"/>
-    </row>
-    <row r="730" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A730" s="35"/>
-    </row>
-    <row r="731" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A731" s="35"/>
-    </row>
-    <row r="732" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A732" s="35"/>
-    </row>
-    <row r="733" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A733" s="35"/>
-    </row>
-    <row r="734" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A734" s="35"/>
-    </row>
-    <row r="735" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A735" s="35"/>
-    </row>
-    <row r="736" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A736" s="35"/>
-    </row>
-    <row r="737" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A737" s="35"/>
-    </row>
-    <row r="738" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A738" s="35"/>
-    </row>
-    <row r="739" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A739" s="35"/>
-    </row>
-    <row r="740" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A740" s="35"/>
-    </row>
-    <row r="741" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A741" s="35"/>
-    </row>
-    <row r="742" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A742" s="35"/>
-    </row>
-    <row r="743" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A743" s="35"/>
-    </row>
-    <row r="744" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A744" s="35"/>
-    </row>
-    <row r="745" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A745" s="35"/>
-    </row>
-    <row r="746" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A746" s="35"/>
-    </row>
-    <row r="747" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A747" s="35"/>
-    </row>
-    <row r="748" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A748" s="35"/>
-    </row>
-    <row r="749" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A749" s="35"/>
-    </row>
-    <row r="750" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A750" s="35"/>
-    </row>
-    <row r="751" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A751" s="35"/>
-    </row>
-    <row r="752" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A752" s="35"/>
-    </row>
-    <row r="753" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A753" s="35"/>
-    </row>
-    <row r="754" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A754" s="35"/>
-    </row>
-    <row r="755" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A755" s="35"/>
-    </row>
-    <row r="756" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A756" s="35"/>
-    </row>
-    <row r="757" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A757" s="35"/>
-    </row>
-    <row r="758" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A758" s="35"/>
-    </row>
-    <row r="759" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A759" s="35"/>
-    </row>
-    <row r="760" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A760" s="35"/>
-    </row>
-    <row r="761" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A761" s="35"/>
-    </row>
-    <row r="762" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A762" s="35"/>
-    </row>
-    <row r="763" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A763" s="35"/>
-    </row>
-    <row r="764" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A764" s="35"/>
-    </row>
-    <row r="765" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A765" s="35"/>
-    </row>
-    <row r="766" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A766" s="35"/>
-    </row>
-    <row r="767" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A767" s="35"/>
-    </row>
-    <row r="768" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A768" s="35"/>
-    </row>
-    <row r="769" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A769" s="35"/>
-    </row>
-    <row r="770" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A770" s="35"/>
-    </row>
-    <row r="771" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A771" s="35"/>
-    </row>
-    <row r="772" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A772" s="35"/>
-    </row>
-    <row r="773" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A773" s="35"/>
-    </row>
-    <row r="774" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A774" s="35"/>
-    </row>
-    <row r="775" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A775" s="35"/>
-    </row>
-    <row r="776" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A776" s="35"/>
-    </row>
-    <row r="777" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A777" s="35"/>
-    </row>
-    <row r="778" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A778" s="35"/>
-    </row>
-    <row r="779" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A779" s="35"/>
-    </row>
-    <row r="780" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A780" s="35"/>
-    </row>
-    <row r="781" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A781" s="35"/>
-    </row>
-    <row r="782" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A782" s="35"/>
-    </row>
-    <row r="783" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A783" s="35"/>
-    </row>
-    <row r="784" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A784" s="35"/>
-    </row>
-    <row r="785" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A785" s="35"/>
-    </row>
-    <row r="786" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A786" s="35"/>
-    </row>
-    <row r="787" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A787" s="35"/>
-    </row>
-    <row r="788" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A788" s="35"/>
-    </row>
-    <row r="789" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A789" s="35"/>
-    </row>
-    <row r="790" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A790" s="35"/>
-    </row>
-    <row r="791" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A791" s="35"/>
-    </row>
-    <row r="792" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A792" s="35"/>
-    </row>
-    <row r="793" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A793" s="35"/>
-    </row>
-    <row r="794" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A794" s="35"/>
-    </row>
-    <row r="795" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A795" s="35"/>
-    </row>
-    <row r="796" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A796" s="35"/>
-    </row>
-    <row r="797" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A797" s="35"/>
-    </row>
-    <row r="798" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A798" s="35"/>
-    </row>
-    <row r="799" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A799" s="35"/>
-    </row>
-    <row r="800" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A800" s="35"/>
-    </row>
-    <row r="801" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A801" s="35"/>
-    </row>
-    <row r="802" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A802" s="35"/>
-    </row>
-    <row r="803" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A803" s="35"/>
-    </row>
-    <row r="804" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A804" s="35"/>
-    </row>
-    <row r="805" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A805" s="35"/>
-    </row>
-    <row r="806" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A806" s="35"/>
-    </row>
-    <row r="807" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A807" s="35"/>
-    </row>
-    <row r="808" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A808" s="35"/>
-    </row>
-    <row r="809" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A809" s="35"/>
-    </row>
-    <row r="810" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A810" s="35"/>
-    </row>
-    <row r="811" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A811" s="35"/>
-    </row>
-    <row r="812" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A812" s="35"/>
-    </row>
-    <row r="813" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A813" s="35"/>
-    </row>
-    <row r="814" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A814" s="35"/>
-    </row>
-    <row r="815" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A815" s="35"/>
-    </row>
-    <row r="816" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A816" s="35"/>
-    </row>
-    <row r="817" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A817" s="35"/>
-    </row>
-    <row r="818" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A818" s="35"/>
-    </row>
-    <row r="819" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A819" s="35"/>
-    </row>
-    <row r="820" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A820" s="35"/>
-    </row>
-    <row r="821" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A821" s="35"/>
-    </row>
-    <row r="822" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A822" s="35"/>
-    </row>
-    <row r="823" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A823" s="35"/>
-    </row>
-    <row r="824" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A824" s="35"/>
-    </row>
-    <row r="825" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A825" s="35"/>
-    </row>
-    <row r="826" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A826" s="35"/>
-    </row>
-    <row r="827" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A827" s="35"/>
-    </row>
-    <row r="828" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A828" s="35"/>
-    </row>
-    <row r="829" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A829" s="35"/>
-    </row>
-    <row r="830" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A830" s="35"/>
-    </row>
-    <row r="831" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A831" s="35"/>
-    </row>
-    <row r="832" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A832" s="35"/>
-    </row>
-    <row r="833" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A833" s="35"/>
-    </row>
-    <row r="834" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A834" s="35"/>
-    </row>
-    <row r="835" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A835" s="35"/>
-    </row>
-    <row r="836" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A836" s="35"/>
-    </row>
-    <row r="837" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A837" s="35"/>
-    </row>
-    <row r="838" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A838" s="35"/>
-    </row>
-    <row r="839" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A839" s="35"/>
-    </row>
-    <row r="840" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A840" s="35"/>
-    </row>
-    <row r="841" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A841" s="35"/>
-    </row>
-    <row r="842" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A842" s="35"/>
-    </row>
-    <row r="843" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A843" s="35"/>
-    </row>
-    <row r="844" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A844" s="35"/>
-    </row>
-    <row r="845" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A845" s="35"/>
-    </row>
-    <row r="846" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A846" s="35"/>
-    </row>
-    <row r="847" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A847" s="35"/>
-    </row>
-    <row r="848" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A848" s="35"/>
-    </row>
-    <row r="849" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A849" s="35"/>
-    </row>
-    <row r="850" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A850" s="35"/>
-    </row>
-    <row r="851" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A851" s="35"/>
-    </row>
-    <row r="852" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A852" s="35"/>
-    </row>
-    <row r="853" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A853" s="35"/>
-    </row>
-    <row r="854" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A854" s="35"/>
-    </row>
-    <row r="855" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A855" s="35"/>
-    </row>
-    <row r="856" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A856" s="35"/>
-    </row>
-    <row r="857" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A857" s="35"/>
-    </row>
-    <row r="858" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A858" s="35"/>
-    </row>
-    <row r="859" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A859" s="35"/>
-    </row>
-    <row r="860" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A860" s="35"/>
-    </row>
-    <row r="861" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A861" s="35"/>
-    </row>
-    <row r="862" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A862" s="35"/>
-    </row>
-    <row r="863" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A863" s="35"/>
-    </row>
-    <row r="864" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A864" s="35"/>
-    </row>
-    <row r="865" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A865" s="35"/>
-    </row>
-    <row r="866" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A866" s="35"/>
-    </row>
-    <row r="867" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A867" s="35"/>
-    </row>
-    <row r="868" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A868" s="35"/>
-    </row>
-    <row r="869" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A869" s="35"/>
-    </row>
-    <row r="870" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A870" s="35"/>
-    </row>
-    <row r="871" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A871" s="35"/>
-    </row>
-    <row r="872" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A872" s="35"/>
-    </row>
-    <row r="873" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A873" s="35"/>
-    </row>
-    <row r="874" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A874" s="35"/>
-    </row>
-    <row r="875" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A875" s="35"/>
-    </row>
-    <row r="876" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A876" s="35"/>
-    </row>
-    <row r="877" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A877" s="35"/>
-    </row>
-    <row r="878" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A878" s="35"/>
-    </row>
-    <row r="879" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A879" s="35"/>
-    </row>
-    <row r="880" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A880" s="35"/>
-    </row>
-    <row r="881" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A881" s="35"/>
-    </row>
-    <row r="882" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A882" s="35"/>
-    </row>
-    <row r="883" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A883" s="35"/>
-    </row>
-    <row r="884" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A884" s="35"/>
-    </row>
-    <row r="885" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A885" s="35"/>
-    </row>
-    <row r="886" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A886" s="35"/>
-    </row>
-    <row r="887" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A887" s="35"/>
-    </row>
-    <row r="888" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A888" s="35"/>
-    </row>
-    <row r="889" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A889" s="35"/>
-    </row>
-    <row r="890" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A890" s="35"/>
-    </row>
-    <row r="891" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A891" s="35"/>
-    </row>
-    <row r="892" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A892" s="35"/>
-    </row>
-    <row r="893" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A893" s="35"/>
-    </row>
-    <row r="894" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A894" s="35"/>
-    </row>
-    <row r="895" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A895" s="35"/>
-    </row>
-    <row r="896" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A896" s="35"/>
-    </row>
-    <row r="897" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A897" s="35"/>
-    </row>
-    <row r="898" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A898" s="35"/>
-    </row>
-    <row r="899" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A899" s="35"/>
-    </row>
-    <row r="900" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A900" s="35"/>
-    </row>
-    <row r="901" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A901" s="35"/>
-    </row>
-    <row r="902" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A902" s="35"/>
-    </row>
-    <row r="903" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A903" s="35"/>
-    </row>
-    <row r="904" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A904" s="35"/>
-    </row>
-    <row r="905" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A905" s="35"/>
-    </row>
-    <row r="906" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A906" s="35"/>
-    </row>
-    <row r="907" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A907" s="35"/>
-    </row>
-    <row r="908" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A908" s="35"/>
-    </row>
-    <row r="909" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A909" s="35"/>
-    </row>
-    <row r="910" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A910" s="35"/>
-    </row>
-    <row r="911" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A911" s="35"/>
-    </row>
-    <row r="912" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A912" s="35"/>
-    </row>
-    <row r="913" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A913" s="35"/>
-    </row>
-    <row r="914" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A914" s="35"/>
-    </row>
-    <row r="915" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A915" s="35"/>
-    </row>
-    <row r="916" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A916" s="35"/>
-    </row>
-    <row r="917" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A917" s="35"/>
-    </row>
-    <row r="918" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A918" s="35"/>
-    </row>
-    <row r="919" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A919" s="35"/>
-    </row>
-    <row r="920" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A920" s="35"/>
-    </row>
-    <row r="921" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A921" s="35"/>
-    </row>
-    <row r="922" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A922" s="35"/>
-    </row>
-    <row r="923" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A923" s="35"/>
-    </row>
-    <row r="924" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A924" s="35"/>
-    </row>
-    <row r="925" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A925" s="35"/>
-    </row>
-    <row r="926" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A926" s="35"/>
-    </row>
-    <row r="927" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A927" s="35"/>
-    </row>
-    <row r="928" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A928" s="35"/>
-    </row>
-    <row r="929" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A929" s="35"/>
-    </row>
-    <row r="930" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A930" s="35"/>
-    </row>
-    <row r="931" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A931" s="35"/>
-    </row>
-    <row r="932" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A932" s="35"/>
-    </row>
-    <row r="933" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A933" s="35"/>
-    </row>
-    <row r="934" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A934" s="35"/>
-    </row>
-    <row r="935" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A935" s="35"/>
-    </row>
-    <row r="936" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A936" s="35"/>
-    </row>
-    <row r="937" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A937" s="35"/>
-    </row>
-    <row r="938" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A938" s="35"/>
-    </row>
-    <row r="939" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A939" s="35"/>
-    </row>
-    <row r="940" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A940" s="35"/>
-    </row>
-    <row r="941" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A941" s="35"/>
-    </row>
-    <row r="942" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A942" s="35"/>
-    </row>
-    <row r="943" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A943" s="35"/>
-    </row>
-    <row r="944" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A944" s="35"/>
-    </row>
-    <row r="945" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A945" s="35"/>
-    </row>
-    <row r="946" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A946" s="35"/>
-    </row>
-    <row r="947" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A947" s="35"/>
-    </row>
-    <row r="948" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A948" s="35"/>
-    </row>
-    <row r="949" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A949" s="35"/>
-    </row>
-    <row r="950" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A950" s="35"/>
-    </row>
-    <row r="951" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A951" s="35"/>
-    </row>
-    <row r="952" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A952" s="35"/>
-    </row>
-    <row r="953" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A953" s="35"/>
-    </row>
-    <row r="954" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A954" s="35"/>
-    </row>
-    <row r="955" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A955" s="35"/>
-    </row>
-    <row r="956" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A956" s="35"/>
-    </row>
-    <row r="957" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A957" s="35"/>
-    </row>
-    <row r="958" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A958" s="35"/>
-    </row>
-    <row r="959" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A959" s="35"/>
-    </row>
-    <row r="960" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A960" s="35"/>
-    </row>
-    <row r="961" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A961" s="35"/>
-    </row>
-    <row r="962" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A962" s="35"/>
-    </row>
-    <row r="963" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A963" s="35"/>
-    </row>
-    <row r="964" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A964" s="35"/>
-    </row>
-    <row r="965" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A965" s="35"/>
-    </row>
-    <row r="966" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A966" s="35"/>
-    </row>
-    <row r="967" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A967" s="35"/>
-    </row>
-    <row r="968" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A968" s="35"/>
-    </row>
-    <row r="969" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A969" s="35"/>
-    </row>
-    <row r="970" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A970" s="35"/>
-    </row>
-    <row r="971" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A971" s="35"/>
-    </row>
-    <row r="972" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A972" s="35"/>
-    </row>
-    <row r="973" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A973" s="35"/>
-    </row>
-    <row r="974" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A974" s="35"/>
-    </row>
-    <row r="975" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A975" s="35"/>
-    </row>
-    <row r="976" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A976" s="35"/>
-    </row>
-    <row r="977" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A977" s="35"/>
-    </row>
-    <row r="978" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A978" s="35"/>
-    </row>
-    <row r="979" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A979" s="35"/>
-    </row>
-    <row r="980" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A980" s="35"/>
-    </row>
-    <row r="981" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A981" s="35"/>
-    </row>
-    <row r="982" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A982" s="35"/>
-    </row>
-    <row r="983" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A983" s="35"/>
-    </row>
-    <row r="984" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A984" s="35"/>
-    </row>
-    <row r="985" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A985" s="35"/>
-    </row>
-    <row r="986" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A986" s="35"/>
-    </row>
-    <row r="987" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A987" s="35"/>
-    </row>
-    <row r="988" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A988" s="35"/>
-    </row>
-    <row r="989" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A989" s="35"/>
-    </row>
-    <row r="990" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A990" s="35"/>
-    </row>
-    <row r="991" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A991" s="35"/>
-    </row>
-    <row r="992" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A992" s="35"/>
-    </row>
-    <row r="993" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A993" s="35"/>
-    </row>
-    <row r="994" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A994" s="35"/>
-    </row>
-    <row r="995" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A995" s="35"/>
-    </row>
-    <row r="996" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A996" s="35"/>
-    </row>
-    <row r="997" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A997" s="35"/>
-    </row>
-    <row r="998" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A998" s="35"/>
-    </row>
-    <row r="999" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A999" s="35"/>
-    </row>
-    <row r="1000" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1000" s="35"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -43787,40 +40533,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="90" t="s">
+      <c r="A1" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="91"/>
-      <c r="C1" s="91"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="91"/>
-      <c r="H1" s="91"/>
-      <c r="I1" s="91"/>
-      <c r="J1" s="91"/>
-      <c r="K1" s="91"/>
-      <c r="L1" s="91"/>
-      <c r="M1" s="91"/>
-      <c r="N1" s="91"/>
-      <c r="O1" s="91"/>
-      <c r="P1" s="91"/>
-      <c r="Q1" s="92"/>
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="E1" s="85"/>
+      <c r="F1" s="85"/>
+      <c r="G1" s="85"/>
+      <c r="H1" s="85"/>
+      <c r="I1" s="85"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="85"/>
+      <c r="L1" s="85"/>
+      <c r="M1" s="85"/>
+      <c r="N1" s="85"/>
+      <c r="O1" s="85"/>
+      <c r="P1" s="85"/>
+      <c r="Q1" s="86"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
     </row>
     <row r="2" spans="1:19" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="96" t="s">
+      <c r="A2" s="90" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
+      <c r="B2" s="90"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="90"/>
+      <c r="I2" s="90"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
@@ -43831,17 +40577,17 @@
       <c r="S2" s="2"/>
     </row>
     <row r="3" spans="1:19" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="97" t="s">
+      <c r="A3" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="97"/>
-      <c r="C3" s="97"/>
-      <c r="D3" s="97"/>
-      <c r="E3" s="97"/>
-      <c r="F3" s="97"/>
-      <c r="G3" s="97"/>
-      <c r="H3" s="97"/>
-      <c r="I3" s="97"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="91"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -43898,11 +40644,11 @@
       <c r="B6" s="10">
         <v>16.5</v>
       </c>
-      <c r="C6" s="86" t="s">
+      <c r="C6" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="87"/>
-      <c r="E6" s="87"/>
+      <c r="D6" s="81"/>
+      <c r="E6" s="81"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
@@ -43918,9 +40664,9 @@
       <c r="B7" s="10">
         <v>5.5</v>
       </c>
-      <c r="C7" s="87"/>
-      <c r="D7" s="87"/>
-      <c r="E7" s="87"/>
+      <c r="C7" s="81"/>
+      <c r="D7" s="81"/>
+      <c r="E7" s="81"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
@@ -43937,9 +40683,9 @@
         <f>SUM(B6:B7)</f>
         <v>22</v>
       </c>
-      <c r="C8" s="87"/>
-      <c r="D8" s="87"/>
-      <c r="E8" s="87"/>
+      <c r="C8" s="81"/>
+      <c r="D8" s="81"/>
+      <c r="E8" s="81"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
@@ -43955,9 +40701,9 @@
       <c r="B9" s="10">
         <v>20</v>
       </c>
-      <c r="C9" s="87"/>
-      <c r="D9" s="87"/>
-      <c r="E9" s="87"/>
+      <c r="C9" s="81"/>
+      <c r="D9" s="81"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
@@ -43981,12 +40727,12 @@
       <c r="L10" s="8"/>
     </row>
     <row r="11" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="93" t="s">
+      <c r="A11" s="87" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="92"/>
+      <c r="B11" s="85"/>
+      <c r="C11" s="85"/>
+      <c r="D11" s="86"/>
       <c r="E11" s="12"/>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
@@ -44050,7 +40796,7 @@
       <c r="C15" s="17">
         <v>0.5</v>
       </c>
-      <c r="D15" s="94">
+      <c r="D15" s="88">
         <v>40</v>
       </c>
     </row>
@@ -44064,7 +40810,7 @@
       <c r="C16" s="17">
         <v>1</v>
       </c>
-      <c r="D16" s="95"/>
+      <c r="D16" s="89"/>
     </row>
     <row r="17" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="15" t="s">
@@ -44087,12 +40833,12 @@
       <c r="D18" s="12"/>
     </row>
     <row r="19" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="83" t="s">
+      <c r="A19" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="84"/>
-      <c r="C19" s="84"/>
-      <c r="D19" s="85"/>
+      <c r="B19" s="78"/>
+      <c r="C19" s="78"/>
+      <c r="D19" s="79"/>
     </row>
     <row r="20" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
@@ -44133,18 +40879,18 @@
         <f>COUNTIF('Sample IDs'!B2:M9,"&lt;&gt;"&amp;"")</f>
         <v>0</v>
       </c>
-      <c r="C24" s="86" t="s">
+      <c r="C24" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="87"/>
-      <c r="E24" s="87"/>
-      <c r="F24" s="87"/>
-      <c r="G24" s="87"/>
-      <c r="H24" s="87"/>
-      <c r="I24" s="87"/>
-      <c r="J24" s="87"/>
-      <c r="K24" s="87"/>
-      <c r="L24" s="87"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="81"/>
+      <c r="G24" s="81"/>
+      <c r="H24" s="81"/>
+      <c r="I24" s="81"/>
+      <c r="J24" s="81"/>
+      <c r="K24" s="81"/>
+      <c r="L24" s="81"/>
     </row>
     <row r="25" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="23" t="s">
@@ -44181,10 +40927,10 @@
       <c r="L26" s="8"/>
     </row>
     <row r="27" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="88" t="s">
+      <c r="A27" s="82" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="89"/>
+      <c r="B27" s="83"/>
       <c r="C27" s="25"/>
       <c r="D27" s="25"/>
       <c r="E27" s="12"/>
@@ -45287,9 +42033,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:O1000"/>
+  <dimension ref="A1:N1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -45304,59 +42050,55 @@
     <col min="10" max="10" width="18.42578125" customWidth="1"/>
     <col min="11" max="11" width="21.5703125" customWidth="1"/>
     <col min="12" max="12" width="60.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="30" width="10.5703125" customWidth="1"/>
+    <col min="13" max="13" width="21.85546875" customWidth="1"/>
+    <col min="14" max="29" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="78" t="s">
+    <row r="1" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="79" t="s">
+      <c r="B1" s="74" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="79" t="s">
+      <c r="C1" s="74" t="s">
         <v>105</v>
       </c>
-      <c r="D1" s="78" t="s">
-        <v>200</v>
+      <c r="D1" s="73" t="s">
+        <v>188</v>
       </c>
-      <c r="E1" s="79" t="s">
-        <v>203</v>
+      <c r="E1" s="74" t="s">
+        <v>191</v>
       </c>
-      <c r="F1" s="78" t="s">
+      <c r="F1" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="79" t="s">
+      <c r="G1" s="74" t="s">
         <v>83</v>
       </c>
-      <c r="H1" s="78" t="s">
+      <c r="H1" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="78" t="s">
+      <c r="I1" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="J1" s="79" t="s">
+      <c r="J1" s="74" t="s">
         <v>87</v>
       </c>
-      <c r="K1" s="78" t="s">
+      <c r="K1" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="L1" s="78" t="s">
+      <c r="L1" s="73" t="s">
         <v>55</v>
       </c>
-      <c r="M1" s="79" t="s">
+      <c r="M1" s="74" t="s">
         <v>134</v>
       </c>
-      <c r="N1" s="79" t="s">
-        <v>152</v>
+      <c r="N1" s="74" t="s">
+        <v>195</v>
       </c>
-      <c r="O1" s="79" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="66" t="s">
         <v>138</v>
       </c>
@@ -45393,28 +42135,25 @@
       <c r="L2" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="M2" s="80" t="s">
+      <c r="M2" s="75" t="s">
         <v>135</v>
       </c>
       <c r="N2" s="66" t="s">
         <v>140</v>
       </c>
-      <c r="O2" s="66" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="66" t="s">
         <v>139</v>
       </c>
       <c r="B3" s="66" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="C3" s="66" t="s">
         <v>98</v>
       </c>
       <c r="D3" s="66" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="E3" s="66" t="s">
         <v>74</v>
@@ -45438,30 +42177,27 @@
         <v>61</v>
       </c>
       <c r="L3" s="66" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
-      <c r="M3" s="80" t="s">
+      <c r="M3" s="75" t="s">
         <v>136</v>
       </c>
       <c r="N3" s="66" t="s">
-        <v>153</v>
+        <v>196</v>
       </c>
-      <c r="O3" s="66" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="81" t="s">
+      <c r="B4" s="76" t="s">
         <v>101</v>
       </c>
       <c r="C4" s="66" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="D4" s="66" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="E4" s="66" t="s">
         <v>73</v>
@@ -45485,17 +42221,14 @@
         <v>103</v>
       </c>
       <c r="L4" s="66" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="M4" s="66"/>
       <c r="N4" s="66" t="s">
-        <v>154</v>
+        <v>197</v>
       </c>
-      <c r="O4" s="66" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="66"/>
       <c r="B5" s="66" t="s">
         <v>62</v>
@@ -45504,7 +42237,7 @@
         <v>99</v>
       </c>
       <c r="D5" s="66" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="E5" s="66" t="s">
         <v>79</v>
@@ -45524,26 +42257,23 @@
         <v>69</v>
       </c>
       <c r="L5" s="66" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="M5" s="66"/>
       <c r="N5" s="66" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
-      <c r="O5" s="66" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="66"/>
       <c r="B6" s="66" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="C6" s="66" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="66" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="E6" s="66" t="s">
         <v>69</v>
@@ -45559,20 +42289,17 @@
       <c r="J6" s="66"/>
       <c r="K6" s="66"/>
       <c r="L6" s="66" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="M6" s="66"/>
       <c r="N6" s="66" t="s">
-        <v>155</v>
+        <v>199</v>
       </c>
-      <c r="O6" s="66" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="66"/>
-      <c r="B7" s="81" t="s">
-        <v>159</v>
+      <c r="B7" s="76" t="s">
+        <v>149</v>
       </c>
       <c r="C7" s="66"/>
       <c r="D7" s="66" t="s">
@@ -45590,20 +42317,17 @@
       <c r="J7" s="66"/>
       <c r="K7" s="66"/>
       <c r="L7" s="66" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="M7" s="66"/>
       <c r="N7" s="66" t="s">
-        <v>156</v>
-      </c>
-      <c r="O7" s="66" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="66"/>
       <c r="B8" s="66" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="C8" s="66"/>
       <c r="D8" s="66" t="s">
@@ -45621,17 +42345,14 @@
       <c r="J8" s="66"/>
       <c r="K8" s="66"/>
       <c r="L8" s="66" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="M8" s="66"/>
-      <c r="N8" s="66" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="66"/>
       <c r="B9" s="66" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="C9" s="66"/>
       <c r="D9" s="66" t="s">
@@ -45649,21 +42370,18 @@
       <c r="J9" s="66"/>
       <c r="K9" s="66"/>
       <c r="L9" s="66" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="M9" s="66"/>
-      <c r="N9" s="66" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="66"/>
-      <c r="B10" s="81" t="s">
-        <v>168</v>
+      <c r="B10" s="76" t="s">
+        <v>158</v>
       </c>
       <c r="C10" s="66"/>
       <c r="D10" s="66" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="E10" s="66"/>
       <c r="F10" s="66" t="s">
@@ -45675,17 +42393,14 @@
       <c r="J10" s="66"/>
       <c r="K10" s="66"/>
       <c r="L10" s="66" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="M10" s="66"/>
-      <c r="N10" s="66" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="66"/>
-      <c r="B11" s="81" t="s">
-        <v>169</v>
+      <c r="B11" s="76" t="s">
+        <v>159</v>
       </c>
       <c r="C11" s="66"/>
       <c r="D11" s="66" t="s">
@@ -45699,19 +42414,18 @@
       <c r="J11" s="66"/>
       <c r="K11" s="66"/>
       <c r="L11" s="66" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="M11" s="66"/>
-      <c r="N11" s="66"/>
-    </row>
-    <row r="12" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="66"/>
       <c r="B12" s="66" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="C12" s="66"/>
       <c r="D12" s="66" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="E12" s="66"/>
       <c r="F12" s="66"/>
@@ -45721,19 +42435,18 @@
       <c r="J12" s="66"/>
       <c r="K12" s="66"/>
       <c r="L12" s="66" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="M12" s="66"/>
-      <c r="N12" s="66"/>
-    </row>
-    <row r="13" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="66"/>
       <c r="B13" s="66" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="C13" s="66"/>
       <c r="D13" s="66" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="E13" s="66"/>
       <c r="F13" s="66"/>
@@ -45743,19 +42456,18 @@
       <c r="J13" s="66"/>
       <c r="K13" s="66"/>
       <c r="L13" s="66" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="M13" s="66"/>
-      <c r="N13" s="66"/>
-    </row>
-    <row r="14" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="66"/>
       <c r="B14" s="66" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="C14" s="66"/>
       <c r="D14" s="66" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="E14" s="66"/>
       <c r="F14" s="66"/>
@@ -45765,15 +42477,14 @@
       <c r="J14" s="66"/>
       <c r="K14" s="66"/>
       <c r="L14" s="66" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="M14" s="66"/>
-      <c r="N14" s="66"/>
-    </row>
-    <row r="15" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="66"/>
       <c r="B15" s="66" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="C15" s="66"/>
       <c r="D15" s="66" t="s">
@@ -45787,19 +42498,18 @@
       <c r="J15" s="66"/>
       <c r="K15" s="66"/>
       <c r="L15" s="66" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="M15" s="66"/>
-      <c r="N15" s="66"/>
-    </row>
-    <row r="16" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="66"/>
       <c r="B16" s="66" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="C16" s="66"/>
       <c r="D16" s="66" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="E16" s="66"/>
       <c r="F16" s="66"/>
@@ -45809,19 +42519,18 @@
       <c r="J16" s="66"/>
       <c r="K16" s="66"/>
       <c r="L16" s="66" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="M16" s="66"/>
-      <c r="N16" s="66"/>
-    </row>
-    <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="66"/>
       <c r="B17" s="66" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C17" s="66"/>
       <c r="D17" s="66" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E17" s="66"/>
       <c r="F17" s="66"/>
@@ -45834,11 +42543,10 @@
         <v>72</v>
       </c>
       <c r="M17" s="66"/>
-      <c r="N17" s="66"/>
-    </row>
-    <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="66"/>
-      <c r="B18" s="81" t="s">
+      <c r="B18" s="76" t="s">
         <v>100</v>
       </c>
       <c r="C18" s="66"/>
@@ -45856,12 +42564,11 @@
         <v>143</v>
       </c>
       <c r="M18" s="66"/>
-      <c r="N18" s="66"/>
-    </row>
-    <row r="19" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="66"/>
       <c r="B19" s="66" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C19" s="66"/>
       <c r="D19" s="66" t="s">
@@ -45875,12 +42582,11 @@
       <c r="J19" s="66"/>
       <c r="K19" s="66"/>
       <c r="M19" s="66"/>
-      <c r="N19" s="66"/>
-    </row>
-    <row r="20" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="66"/>
       <c r="B20" s="66" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C20" s="66"/>
       <c r="D20" s="66" t="s">
@@ -45894,12 +42600,11 @@
       <c r="J20" s="66"/>
       <c r="K20" s="66"/>
       <c r="M20" s="66"/>
-      <c r="N20" s="66"/>
-    </row>
-    <row r="21" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="66"/>
-      <c r="B21" s="81" t="s">
-        <v>160</v>
+      <c r="B21" s="76" t="s">
+        <v>150</v>
       </c>
       <c r="C21" s="66"/>
       <c r="D21" s="66" t="s">
@@ -45914,12 +42619,11 @@
       <c r="K21" s="66"/>
       <c r="L21" s="66"/>
       <c r="M21" s="66"/>
-      <c r="N21" s="66"/>
-    </row>
-    <row r="22" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="66"/>
-      <c r="B22" s="81" t="s">
-        <v>172</v>
+      <c r="B22" s="76" t="s">
+        <v>162</v>
       </c>
       <c r="C22" s="66"/>
       <c r="D22" s="66" t="s">
@@ -45934,12 +42638,11 @@
       <c r="K22" s="66"/>
       <c r="L22" s="66"/>
       <c r="M22" s="66"/>
-      <c r="N22" s="66"/>
-    </row>
-    <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="66"/>
-      <c r="B23" s="81" t="s">
-        <v>174</v>
+      <c r="B23" s="76" t="s">
+        <v>164</v>
       </c>
       <c r="C23" s="66"/>
       <c r="D23" s="66" t="s">
@@ -45954,12 +42657,11 @@
       <c r="K23" s="66"/>
       <c r="L23" s="66"/>
       <c r="M23" s="66"/>
-      <c r="N23" s="66"/>
-    </row>
-    <row r="24" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="66"/>
-      <c r="B24" s="81" t="s">
-        <v>173</v>
+      <c r="B24" s="76" t="s">
+        <v>163</v>
       </c>
       <c r="C24" s="66"/>
       <c r="D24" s="66" t="s">
@@ -45974,12 +42676,11 @@
       <c r="K24" s="66"/>
       <c r="L24" s="66"/>
       <c r="M24" s="66"/>
-      <c r="N24" s="66"/>
-    </row>
-    <row r="25" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="66"/>
-      <c r="B25" s="81" t="s">
-        <v>171</v>
+      <c r="B25" s="76" t="s">
+        <v>161</v>
       </c>
       <c r="C25" s="66"/>
       <c r="D25" s="66" t="s">
@@ -45994,17 +42695,16 @@
       <c r="K25" s="66"/>
       <c r="L25" s="66"/>
       <c r="M25" s="66"/>
-      <c r="N25" s="66"/>
-    </row>
-    <row r="26" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="66" t="s">
         <v>71</v>
       </c>
       <c r="D26" s="66" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="66" t="s">
         <v>69</v>
       </c>
@@ -46012,11 +42712,11 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>